<commit_message>
updated all input/output paths
</commit_message>
<xml_diff>
--- a/Input/Names_variations.xlsx
+++ b/Input/Names_variations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Media-Monitoring\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7543F231-DFEE-4BC9-A34C-746E1180B159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57CE109-E025-4EDC-B308-38F8124331AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devendra Fadnavis" sheetId="1" r:id="rId1"/>

</xml_diff>